<commit_message>
Perform more excel function
</commit_message>
<xml_diff>
--- a/Superstore data.xlsx
+++ b/Superstore data.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Project\Sales and profit analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBECD66-C657-4CEB-9D6C-FEA25BDD4801}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17A5A6F-36C4-485C-9A9E-0919A9258DB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Full data" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="5" r:id="rId2"/>
+    <sheet name="Summery" sheetId="5" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Full data'!$A$1:$O$1</definedName>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="179">
   <si>
     <t>Order ID</t>
   </si>
@@ -593,13 +593,16 @@
   </si>
   <si>
     <t>Using Vlookup Find perticular details</t>
+  </si>
+  <si>
+    <t>Using Xlookup Find perticular details</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -644,6 +647,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Arial"/>
@@ -651,7 +663,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -694,6 +706,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -731,7 +761,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -750,28 +780,46 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2533,7 +2581,7 @@
       </c>
     </row>
     <row r="32" spans="1:15" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="7" t="s">
         <v>136</v>
       </c>
       <c r="B32" s="4">
@@ -2721,7 +2769,7 @@
       </c>
     </row>
     <row r="36" spans="1:15" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="7" t="s">
         <v>154</v>
       </c>
       <c r="B36" s="4">
@@ -6841,15 +6889,15 @@
   </sheetData>
   <autoFilter ref="A1:O1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="N2:N41">
-    <cfRule type="cellIs" dxfId="6" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="greaterThan">
       <formula>0.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="greaterThan">
       <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O1:O1048576">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6859,11 +6907,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B17FDCDB-B318-4851-8D50-A72FD6AB6F05}">
-  <dimension ref="B1:AF12"/>
+  <dimension ref="B1:AV12"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
@@ -6877,39 +6925,53 @@
     <col min="15" max="15" width="5" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="6" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="59.5546875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="2" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="8" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="8" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="15" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="10.77734375" style="6" customWidth="1"/>
+    <col min="36" max="36" width="10.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="59.5546875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="8" bestFit="1" customWidth="1"/>
+    <col min="46" max="47" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:32" x14ac:dyDescent="0.25">
-      <c r="B1" s="10" t="s">
+    <row r="1" spans="2:48" x14ac:dyDescent="0.25">
+      <c r="B1" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="R1" s="11" t="s">
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="R1" s="12" t="s">
         <v>177</v>
       </c>
       <c r="S1" s="12"/>
@@ -6926,108 +6988,170 @@
       <c r="AD1" s="12"/>
       <c r="AE1" s="12"/>
       <c r="AF1" s="12"/>
-    </row>
-    <row r="2" spans="2:32" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+      <c r="AH1" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="AI1" s="21"/>
+      <c r="AJ1" s="21"/>
+      <c r="AK1" s="21"/>
+      <c r="AL1" s="21"/>
+      <c r="AM1" s="21"/>
+      <c r="AN1" s="21"/>
+      <c r="AO1" s="21"/>
+      <c r="AP1" s="21"/>
+      <c r="AQ1" s="21"/>
+      <c r="AR1" s="21"/>
+      <c r="AS1" s="21"/>
+      <c r="AT1" s="21"/>
+      <c r="AU1" s="21"/>
+      <c r="AV1" s="21"/>
+    </row>
+    <row r="2" spans="2:48" x14ac:dyDescent="0.25">
+      <c r="B2" s="14" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="M2" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="N2" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="O2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="P2" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="R2" s="13" t="s">
+      <c r="R2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="S2" s="14" t="s">
+      <c r="S2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="T2" s="15" t="s">
+      <c r="T2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="U2" s="13" t="s">
+      <c r="U2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="V2" s="13" t="s">
+      <c r="V2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="W2" s="13" t="s">
+      <c r="W2" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="X2" s="13" t="s">
+      <c r="X2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="Y2" s="13" t="s">
+      <c r="Y2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="Z2" s="13" t="s">
+      <c r="Z2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="AA2" s="13" t="s">
+      <c r="AA2" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="AB2" s="13" t="s">
+      <c r="AB2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="AC2" s="13" t="s">
+      <c r="AC2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="AD2" s="13" t="s">
+      <c r="AD2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="AE2" s="13" t="s">
+      <c r="AE2" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="AF2" s="13" t="s">
+      <c r="AF2" s="15" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AH2" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ2" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="AK2" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL2" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="AM2" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="AN2" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="AO2" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="AP2" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="AQ2" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="AR2" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="AS2" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="AT2" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="AU2" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="AV2" s="17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B3" s="9" t="str" cm="1">
         <f t="array" ref="B3:P12">_xlfn._xlws.FILTER('Full data'!A2:O41,'Full data'!O2:O41&lt;0)</f>
         <v>US-2015-108966</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="23">
         <v>42318</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="23">
         <v>42295</v>
       </c>
       <c r="E3" s="9" t="str">
@@ -7069,58 +7193,104 @@
       <c r="R3" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="S3" s="16" cm="1">
+      <c r="S3" s="22" cm="1">
         <f t="array" ref="S3:AF3">VLOOKUP(R3,'Full data'!A2:O41,{2,3,4,5,6,7,8,9,10,11,12,13,14,15},FALSE)</f>
         <v>41888</v>
       </c>
-      <c r="T3" s="16">
+      <c r="T3" s="22">
         <v>41804</v>
       </c>
-      <c r="U3" s="16" t="str">
+      <c r="U3" s="11" t="str">
         <v>Standard Class</v>
       </c>
-      <c r="V3" s="16" t="str">
+      <c r="V3" s="11" t="str">
         <v>BH-11710</v>
       </c>
-      <c r="W3" s="16" t="str">
+      <c r="W3" s="11" t="str">
         <v>Brosina Hoffman</v>
       </c>
-      <c r="X3" s="16" t="str">
+      <c r="X3" s="11" t="str">
         <v>California</v>
       </c>
-      <c r="Y3" s="16" t="str">
+      <c r="Y3" s="11" t="str">
         <v>FUR-FU-10001487</v>
       </c>
-      <c r="Z3" s="16" t="str">
+      <c r="Z3" s="11" t="str">
         <v>Furniture</v>
       </c>
-      <c r="AA3" s="16" t="str">
+      <c r="AA3" s="11" t="str">
         <v>Furnishings</v>
       </c>
-      <c r="AB3" s="16" t="str">
+      <c r="AB3" s="11" t="str">
         <v>Eldon Expressions Wood and Plastic Desk Accessories, Cherry Wood</v>
       </c>
-      <c r="AC3" s="16">
+      <c r="AC3" s="11">
         <v>48.86</v>
       </c>
-      <c r="AD3" s="16">
+      <c r="AD3" s="11">
         <v>7</v>
       </c>
-      <c r="AE3" s="16">
+      <c r="AE3" s="11">
         <v>0</v>
       </c>
-      <c r="AF3" s="16">
+      <c r="AF3" s="11">
         <v>14.1694</v>
       </c>
-    </row>
-    <row r="4" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AH3" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="AI3" s="24" cm="1">
+        <f t="array" ref="AI3:AV3">_xlfn.XLOOKUP(AH3,'Full data'!A2:A41,'Full data'!B2:O41,"not found",0)</f>
+        <v>41888</v>
+      </c>
+      <c r="AJ3" s="24">
+        <v>41804</v>
+      </c>
+      <c r="AK3" s="19" t="str">
+        <v>Standard Class</v>
+      </c>
+      <c r="AL3" s="19" t="str">
+        <v>BH-11710</v>
+      </c>
+      <c r="AM3" s="19" t="str">
+        <v>Brosina Hoffman</v>
+      </c>
+      <c r="AN3" s="19" t="str">
+        <v>California</v>
+      </c>
+      <c r="AO3" s="19" t="str">
+        <v>FUR-FU-10001487</v>
+      </c>
+      <c r="AP3" s="19" t="str">
+        <v>Furniture</v>
+      </c>
+      <c r="AQ3" s="19" t="str">
+        <v>Furnishings</v>
+      </c>
+      <c r="AR3" s="19" t="str">
+        <v>Eldon Expressions Wood and Plastic Desk Accessories, Cherry Wood</v>
+      </c>
+      <c r="AS3" s="19">
+        <v>48.86</v>
+      </c>
+      <c r="AT3" s="19">
+        <v>7</v>
+      </c>
+      <c r="AU3" s="19">
+        <v>0</v>
+      </c>
+      <c r="AV3" s="19">
+        <v>14.1694</v>
+      </c>
+    </row>
+    <row r="4" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B4" s="9" t="str">
         <v>US-2015-118983</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="23">
         <v>42330</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="23">
         <v>42334</v>
       </c>
       <c r="E4" s="9" t="str">
@@ -7159,61 +7329,107 @@
       <c r="P4" s="9">
         <v>-123.858</v>
       </c>
-      <c r="R4" s="16" t="s">
+      <c r="R4" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="S4" s="16" cm="1">
+      <c r="S4" s="22" cm="1">
         <f t="array" ref="S4:AF4">VLOOKUP(R4,'Full data'!A3:O42,{2,3,4,5,6,7,8,9,10,11,12,13,14,15},FALSE)</f>
         <v>42264</v>
       </c>
-      <c r="T4" s="16">
+      <c r="T4" s="22">
         <v>42268</v>
       </c>
-      <c r="U4" s="16" t="str">
+      <c r="U4" s="11" t="str">
         <v>Standard Class</v>
       </c>
-      <c r="V4" s="16" t="str">
+      <c r="V4" s="11" t="str">
         <v>TB-21520</v>
       </c>
-      <c r="W4" s="16" t="str">
+      <c r="W4" s="11" t="str">
         <v>Tracy Blumstein</v>
       </c>
-      <c r="X4" s="16" t="str">
+      <c r="X4" s="11" t="str">
         <v>Pennsylvania</v>
       </c>
-      <c r="Y4" s="16" t="str">
+      <c r="Y4" s="11" t="str">
         <v>FUR-BO-10004834</v>
       </c>
-      <c r="Z4" s="16" t="str">
+      <c r="Z4" s="11" t="str">
         <v>Furniture</v>
       </c>
-      <c r="AA4" s="16" t="str">
+      <c r="AA4" s="11" t="str">
         <v>Bookcases</v>
       </c>
-      <c r="AB4" s="16" t="str">
+      <c r="AB4" s="11" t="str">
         <v>Riverside Palais Royal Lawyers Bookcase, Royale Cherry Finish</v>
       </c>
-      <c r="AC4" s="16">
+      <c r="AC4" s="11">
         <v>3083.43</v>
       </c>
-      <c r="AD4" s="16">
+      <c r="AD4" s="11">
         <v>7</v>
       </c>
-      <c r="AE4" s="16">
+      <c r="AE4" s="11">
         <v>0.5</v>
       </c>
-      <c r="AF4" s="16">
+      <c r="AF4" s="11">
         <v>-1665.0522000000001</v>
       </c>
-    </row>
-    <row r="5" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AH4" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="AI4" s="24" cm="1">
+        <f t="array" ref="AI4:AV4">_xlfn.XLOOKUP(AH4,'Full data'!A3:A42,'Full data'!B3:O42,"not found",0)</f>
+        <v>42264</v>
+      </c>
+      <c r="AJ4" s="24">
+        <v>42268</v>
+      </c>
+      <c r="AK4" s="19" t="str">
+        <v>Standard Class</v>
+      </c>
+      <c r="AL4" s="19" t="str">
+        <v>TB-21520</v>
+      </c>
+      <c r="AM4" s="19" t="str">
+        <v>Tracy Blumstein</v>
+      </c>
+      <c r="AN4" s="19" t="str">
+        <v>Pennsylvania</v>
+      </c>
+      <c r="AO4" s="19" t="str">
+        <v>FUR-BO-10004834</v>
+      </c>
+      <c r="AP4" s="19" t="str">
+        <v>Furniture</v>
+      </c>
+      <c r="AQ4" s="19" t="str">
+        <v>Bookcases</v>
+      </c>
+      <c r="AR4" s="19" t="str">
+        <v>Riverside Palais Royal Lawyers Bookcase, Royale Cherry Finish</v>
+      </c>
+      <c r="AS4" s="19">
+        <v>3083.43</v>
+      </c>
+      <c r="AT4" s="19">
+        <v>7</v>
+      </c>
+      <c r="AU4" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="AV4" s="19">
+        <v>-1665.0522000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B5" s="9" t="str">
         <v>US-2015-118983</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="23">
         <v>42330</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="23">
         <v>42334</v>
       </c>
       <c r="E5" s="9" t="str">
@@ -7252,61 +7468,107 @@
       <c r="P5" s="9">
         <v>-3.8159999999999998</v>
       </c>
-      <c r="R5" s="16" t="s">
+      <c r="R5" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="S5" s="16" cm="1">
+      <c r="S5" s="22" cm="1">
         <f t="array" ref="S5:AF5">VLOOKUP(R5,'Full data'!A4:O43,{2,3,4,5,6,7,8,9,10,11,12,13,14,15},FALSE)</f>
         <v>42365</v>
       </c>
-      <c r="T5" s="16">
+      <c r="T5" s="22">
         <v>42369</v>
       </c>
-      <c r="U5" s="16" t="str">
+      <c r="U5" s="11" t="str">
         <v>Standard Class</v>
       </c>
-      <c r="V5" s="16" t="str">
+      <c r="V5" s="11" t="str">
         <v>SN-20710</v>
       </c>
-      <c r="W5" s="16" t="str">
+      <c r="W5" s="11" t="str">
         <v>Steve Nguyen</v>
       </c>
-      <c r="X5" s="16" t="str">
+      <c r="X5" s="11" t="str">
         <v>Texas</v>
       </c>
-      <c r="Y5" s="16" t="str">
+      <c r="Y5" s="11" t="str">
         <v>OFF-EN-10002986</v>
       </c>
-      <c r="Z5" s="16" t="str">
+      <c r="Z5" s="11" t="str">
         <v>Office Supplies</v>
       </c>
-      <c r="AA5" s="16" t="str">
+      <c r="AA5" s="11" t="str">
         <v>Envelopes</v>
       </c>
-      <c r="AB5" s="16" t="str">
+      <c r="AB5" s="11" t="str">
         <v>#10-4 1/8" x 9 1/2" Premium Diagonal Seam Envelopes</v>
       </c>
-      <c r="AC5" s="16">
+      <c r="AC5" s="11">
         <v>113.328</v>
       </c>
-      <c r="AD5" s="16">
+      <c r="AD5" s="11">
         <v>9</v>
       </c>
-      <c r="AE5" s="16">
+      <c r="AE5" s="11">
         <v>0.2</v>
       </c>
-      <c r="AF5" s="16">
+      <c r="AF5" s="11">
         <v>35.414999999999999</v>
       </c>
-    </row>
-    <row r="6" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AH5" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="AI5" s="24" cm="1">
+        <f t="array" ref="AI5:AV5">_xlfn.XLOOKUP(AH5,'Full data'!A4:A43,'Full data'!B4:O43,"not found",0)</f>
+        <v>43027</v>
+      </c>
+      <c r="AJ5" s="24">
+        <v>43031</v>
+      </c>
+      <c r="AK5" s="19" t="str">
+        <v>Second Class</v>
+      </c>
+      <c r="AL5" s="19" t="str">
+        <v>MA-17560</v>
+      </c>
+      <c r="AM5" s="19" t="str">
+        <v>Matt Abelman</v>
+      </c>
+      <c r="AN5" s="19" t="str">
+        <v>Texas</v>
+      </c>
+      <c r="AO5" s="19" t="str">
+        <v>OFF-PA-10000249</v>
+      </c>
+      <c r="AP5" s="19" t="str">
+        <v>Office Supplies</v>
+      </c>
+      <c r="AQ5" s="19" t="str">
+        <v>Paper</v>
+      </c>
+      <c r="AR5" s="19" t="str">
+        <v>Easy-staple paper</v>
+      </c>
+      <c r="AS5" s="19">
+        <v>29.472000000000001</v>
+      </c>
+      <c r="AT5" s="19">
+        <v>3</v>
+      </c>
+      <c r="AU5" s="19">
+        <v>0.2</v>
+      </c>
+      <c r="AV5" s="19">
+        <v>9.9467999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="str">
         <v>US-2017-156909</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="23">
         <v>42932</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="23">
         <v>42934</v>
       </c>
       <c r="E6" s="9" t="str">
@@ -7345,61 +7607,107 @@
       <c r="P6" s="9">
         <v>-1.0196000000000001</v>
       </c>
-      <c r="R6" s="16" t="s">
+      <c r="R6" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="S6" s="16" cm="1">
+      <c r="S6" s="22" cm="1">
         <f t="array" ref="S6:AF6">VLOOKUP(R6,'Full data'!A5:O44,{2,3,4,5,6,7,8,9,10,11,12,13,14,15},FALSE)</f>
         <v>42365</v>
       </c>
-      <c r="T6" s="16">
+      <c r="T6" s="22">
         <v>42369</v>
       </c>
-      <c r="U6" s="16" t="str">
+      <c r="U6" s="11" t="str">
         <v>Standard Class</v>
       </c>
-      <c r="V6" s="16" t="str">
+      <c r="V6" s="11" t="str">
         <v>SN-20710</v>
       </c>
-      <c r="W6" s="16" t="str">
+      <c r="W6" s="11" t="str">
         <v>Steve Nguyen</v>
       </c>
-      <c r="X6" s="16" t="str">
+      <c r="X6" s="11" t="str">
         <v>Texas</v>
       </c>
-      <c r="Y6" s="16" t="str">
+      <c r="Y6" s="11" t="str">
         <v>OFF-EN-10002986</v>
       </c>
-      <c r="Z6" s="16" t="str">
+      <c r="Z6" s="11" t="str">
         <v>Office Supplies</v>
       </c>
-      <c r="AA6" s="16" t="str">
+      <c r="AA6" s="11" t="str">
         <v>Envelopes</v>
       </c>
-      <c r="AB6" s="16" t="str">
+      <c r="AB6" s="11" t="str">
         <v>#10-4 1/8" x 9 1/2" Premium Diagonal Seam Envelopes</v>
       </c>
-      <c r="AC6" s="16">
+      <c r="AC6" s="11">
         <v>113.328</v>
       </c>
-      <c r="AD6" s="16">
+      <c r="AD6" s="11">
         <v>9</v>
       </c>
-      <c r="AE6" s="16">
+      <c r="AE6" s="11">
         <v>0.2</v>
       </c>
-      <c r="AF6" s="16">
+      <c r="AF6" s="11">
         <v>35.414999999999999</v>
       </c>
-    </row>
-    <row r="7" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="AH6" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="AI6" s="24" cm="1">
+        <f t="array" ref="AI6:AV6">_xlfn.XLOOKUP(AH6,'Full data'!A5:A44,'Full data'!B5:O44,"not found",0)</f>
+        <v>42365</v>
+      </c>
+      <c r="AJ6" s="24">
+        <v>42369</v>
+      </c>
+      <c r="AK6" s="19" t="str">
+        <v>Standard Class</v>
+      </c>
+      <c r="AL6" s="19" t="str">
+        <v>SN-20710</v>
+      </c>
+      <c r="AM6" s="19" t="str">
+        <v>Steve Nguyen</v>
+      </c>
+      <c r="AN6" s="19" t="str">
+        <v>Texas</v>
+      </c>
+      <c r="AO6" s="19" t="str">
+        <v>OFF-EN-10002986</v>
+      </c>
+      <c r="AP6" s="19" t="str">
+        <v>Office Supplies</v>
+      </c>
+      <c r="AQ6" s="19" t="str">
+        <v>Envelopes</v>
+      </c>
+      <c r="AR6" s="19" t="str">
+        <v>#10-4 1/8" x 9 1/2" Premium Diagonal Seam Envelopes</v>
+      </c>
+      <c r="AS6" s="19">
+        <v>113.328</v>
+      </c>
+      <c r="AT6" s="19">
+        <v>9</v>
+      </c>
+      <c r="AU6" s="19">
+        <v>0.2</v>
+      </c>
+      <c r="AV6" s="19">
+        <v>35.414999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="str">
         <v>US-2015-150630</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="23">
         <v>42264</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="23">
         <v>42268</v>
       </c>
       <c r="E7" s="9" t="str">
@@ -7439,14 +7747,14 @@
         <v>-1665.0522000000001</v>
       </c>
     </row>
-    <row r="8" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B8" s="9" t="str">
         <v>US-2015-150630</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="23">
         <v>42264</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="23">
         <v>42268</v>
       </c>
       <c r="E8" s="9" t="str">
@@ -7486,14 +7794,14 @@
         <v>-7.0532000000000004</v>
       </c>
     </row>
-    <row r="9" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B9" s="9" t="str">
         <v>US-2015-150630</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="23">
         <v>42264</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="23">
         <v>42268</v>
       </c>
       <c r="E9" s="9" t="str">
@@ -7533,14 +7841,14 @@
         <v>-5.7149999999999999</v>
       </c>
     </row>
-    <row r="10" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B10" s="9" t="str">
         <v>CA-2016-117590</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="23">
         <v>42594</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="23">
         <v>42655</v>
       </c>
       <c r="E10" s="9" t="str">
@@ -7580,14 +7888,14 @@
         <v>-147.96299999999999</v>
       </c>
     </row>
-    <row r="11" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="str">
         <v>CA-2015-117415</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="23">
         <v>42365</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="23">
         <v>42369</v>
       </c>
       <c r="E11" s="9" t="str">
@@ -7627,14 +7935,14 @@
         <v>-46.976399999999998</v>
       </c>
     </row>
-    <row r="12" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="str">
         <v>CA-2015-117415</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="23">
         <v>42365</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="23">
         <v>42369</v>
       </c>
       <c r="E12" s="9" t="str">
@@ -7675,16 +7983,22 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B1:P1"/>
     <mergeCell ref="R1:AF1"/>
+    <mergeCell ref="AH1:AV1"/>
   </mergeCells>
   <conditionalFormatting sqref="P2">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF2">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AV2">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>